<commit_message>
Radar: datos de 2026-08-23
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E29</f>
+        <f>E30</f>
         <v/>
       </c>
     </row>
@@ -1237,10 +1237,10 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="18" t="n">
+      <c r="D28" s="13" t="n">
         <v>46257</v>
       </c>
-      <c r="E28" s="19" t="n">
+      <c r="E28" s="12" t="n">
         <v>66.68000000000001</v>
       </c>
     </row>
@@ -1251,14 +1251,11 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E29" s="21">
-        <f>AVERAGE(E6:E28)</f>
-        <v/>
+      <c r="D29" s="18" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E29" s="19" t="n">
+        <v>66.22</v>
       </c>
     </row>
     <row r="30">
@@ -1268,10 +1265,14 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E30" s="21">
+        <f>AVERAGE(E6:E29)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1281,6 +1282,11 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1522,12 +1528,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D30:H30"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D31:H31"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1537,7 +1543,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E28">
+  <conditionalFormatting sqref="E6:E29">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1821,7 +1827,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E29</f>
+        <f>MIBGAS_Spot!E30</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-24
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E30</f>
+        <f>E31</f>
         <v/>
       </c>
     </row>
@@ -1251,10 +1251,10 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="18" t="n">
+      <c r="D29" s="13" t="n">
         <v>46258</v>
       </c>
-      <c r="E29" s="19" t="n">
+      <c r="E29" s="12" t="n">
         <v>66.22</v>
       </c>
     </row>
@@ -1265,14 +1265,11 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E30" s="21">
-        <f>AVERAGE(E6:E29)</f>
-        <v/>
+      <c r="D30" s="18" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E30" s="19" t="n">
+        <v>67.97</v>
       </c>
     </row>
     <row r="31">
@@ -1282,10 +1279,14 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E31" s="21">
+        <f>AVERAGE(E6:E30)</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -1294,6 +1295,11 @@
       </c>
       <c r="B32" s="12" t="n">
         <v>41.41</v>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1533,7 +1539,7 @@
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="D32:H32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1543,7 +1549,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E29">
+  <conditionalFormatting sqref="E6:E30">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1601,7 +1607,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1633,7 +1639,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>66.04000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1651,7 +1657,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>65.25</v>
+        <v>66.42</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1669,7 +1675,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>66.25</v>
+        <v>67.3</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1687,7 +1693,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>65.87</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1705,7 +1711,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>63.75</v>
+        <v>64.55</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1723,7 +1729,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>44.88</v>
+        <v>44.62</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1736,7 +1742,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>42.01</v>
+        <v>41.57</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1749,7 +1755,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>43.44</v>
+        <v>43.09</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1762,7 +1768,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>64.81999999999999</v>
+        <v>65.73</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1775,7 +1781,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>47.95</v>
+        <v>47.83</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1788,7 +1794,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>32.4</v>
+        <v>31.58</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1827,7 +1833,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E30</f>
+        <f>MIBGAS_Spot!E31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-25
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E31</f>
+        <f>E32</f>
         <v/>
       </c>
     </row>
@@ -1265,10 +1265,10 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="18" t="n">
+      <c r="D30" s="13" t="n">
         <v>46259</v>
       </c>
-      <c r="E30" s="19" t="n">
+      <c r="E30" s="12" t="n">
         <v>67.97</v>
       </c>
     </row>
@@ -1279,14 +1279,11 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E31" s="21">
-        <f>AVERAGE(E6:E30)</f>
-        <v/>
+      <c r="D31" s="18" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E31" s="19" t="n">
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="32">
@@ -1296,10 +1293,14 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E32" s="21">
+        <f>AVERAGE(E6:E31)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1308,6 +1309,11 @@
       </c>
       <c r="B33" s="12" t="n">
         <v>33.76</v>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1537,9 +1543,9 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D33:H33"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D32:H32"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1549,7 +1555,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E30">
+  <conditionalFormatting sqref="E6:E31">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1607,7 +1613,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1639,7 +1645,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>67.3</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1657,7 +1663,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>66.42</v>
+        <v>65.45</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1675,7 +1681,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>67.3</v>
+        <v>65.2</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1693,7 +1699,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>67.34999999999999</v>
+        <v>65.33</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1711,7 +1717,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>64.55</v>
+        <v>62.9</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1729,7 +1735,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>44.62</v>
+        <v>44.03</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1742,7 +1748,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>41.57</v>
+        <v>41.01</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1755,7 +1761,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>43.09</v>
+        <v>42.51</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1768,7 +1774,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>65.73</v>
+        <v>64.13</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1781,7 +1787,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>47.83</v>
+        <v>47.3</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1794,7 +1800,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>31.58</v>
+        <v>31.44</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1833,7 +1839,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E31</f>
+        <f>MIBGAS_Spot!E32</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-26
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E32</f>
+        <f>E33</f>
         <v/>
       </c>
     </row>
@@ -1279,10 +1279,10 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="18" t="n">
+      <c r="D31" s="13" t="n">
         <v>46260</v>
       </c>
-      <c r="E31" s="19" t="n">
+      <c r="E31" s="12" t="n">
         <v>66.09999999999999</v>
       </c>
     </row>
@@ -1293,14 +1293,11 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E32" s="21">
-        <f>AVERAGE(E6:E31)</f>
-        <v/>
+      <c r="D32" s="18" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>65.86</v>
       </c>
     </row>
     <row r="33">
@@ -1310,10 +1307,14 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D33" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E33" s="21">
+        <f>AVERAGE(E6:E32)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1322,6 +1323,11 @@
       </c>
       <c r="B34" s="12" t="n">
         <v>34.02</v>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1542,8 +1548,8 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D34:H34"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D33:H33"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1555,7 +1561,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E31">
+  <conditionalFormatting sqref="E6:E32">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1613,7 +1619,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1645,7 +1651,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>66.59999999999999</v>
+        <v>63.76</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1663,7 +1669,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>65.45</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1681,7 +1687,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>65.2</v>
+        <v>64</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1699,7 +1705,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>65.33</v>
+        <v>63.95</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1717,7 +1723,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>62.9</v>
+        <v>63.33</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1735,7 +1741,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>44.03</v>
+        <v>44.41</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1748,7 +1754,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>41.01</v>
+        <v>41.45</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1761,7 +1767,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>42.51</v>
+        <v>42.93</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1774,7 +1780,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>64.13</v>
+        <v>62.8</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1787,7 +1793,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>47.3</v>
+        <v>47.46</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1800,7 +1806,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>31.44</v>
+        <v>31.81</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1839,7 +1845,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E32</f>
+        <f>MIBGAS_Spot!E33</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-28
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -203,12 +203,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1100,7 +1094,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E33</f>
+        <f>E34</f>
         <v/>
       </c>
     </row>
@@ -1293,10 +1287,10 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="18" t="n">
+      <c r="D32" s="13" t="n">
         <v>46261</v>
       </c>
-      <c r="E32" s="19" t="n">
+      <c r="E32" s="12" t="n">
         <v>65.86</v>
       </c>
     </row>
@@ -1307,14 +1301,11 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E33" s="21">
-        <f>AVERAGE(E6:E32)</f>
-        <v/>
+      <c r="D33" s="13" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>68.38</v>
       </c>
     </row>
     <row r="34">
@@ -1324,10 +1315,14 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E34" s="19">
+        <f>AVERAGE(E6:E33)</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -1337,6 +1332,11 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
+      <c r="D35" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -1446,109 +1446,109 @@
       <c r="A49" s="11" t="n">
         <v>46235</v>
       </c>
-      <c r="B49" s="23" t="n"/>
+      <c r="B49" s="21" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n">
         <v>46266</v>
       </c>
-      <c r="B50" s="23" t="n"/>
+      <c r="B50" s="21" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="B51" s="23" t="n"/>
+      <c r="B51" s="21" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
         <v>46327</v>
       </c>
-      <c r="B52" s="23" t="n"/>
+      <c r="B52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
         <v>46357</v>
       </c>
-      <c r="B53" s="23" t="n"/>
+      <c r="B53" s="21" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
         <v>46388</v>
       </c>
-      <c r="B54" s="23" t="n"/>
+      <c r="B54" s="21" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
         <v>46419</v>
       </c>
-      <c r="B55" s="23" t="n"/>
+      <c r="B55" s="21" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
         <v>46447</v>
       </c>
-      <c r="B56" s="23" t="n"/>
+      <c r="B56" s="21" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
         <v>46478</v>
       </c>
-      <c r="B57" s="23" t="n"/>
+      <c r="B57" s="21" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
         <v>46508</v>
       </c>
-      <c r="B58" s="23" t="n"/>
+      <c r="B58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
         <v>46539</v>
       </c>
-      <c r="B59" s="23" t="n"/>
+      <c r="B59" s="21" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
         <v>46569</v>
       </c>
-      <c r="B60" s="23" t="n"/>
+      <c r="B60" s="21" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
         <v>46600</v>
       </c>
-      <c r="B61" s="23" t="n"/>
+      <c r="B61" s="21" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
         <v>46631</v>
       </c>
-      <c r="B62" s="23" t="n"/>
+      <c r="B62" s="21" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
         <v>46661</v>
       </c>
-      <c r="B63" s="23" t="n"/>
+      <c r="B63" s="21" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
         <v>46692</v>
       </c>
-      <c r="B64" s="23" t="n"/>
+      <c r="B64" s="21" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
         <v>46722</v>
       </c>
-      <c r="B65" s="23" t="n"/>
+      <c r="B65" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D35:H35"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D34:H34"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
@@ -1561,7 +1561,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E32">
+  <conditionalFormatting sqref="E6:E33">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1613,13 +1613,13 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Fecha de la curva:</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
-        <v>46260</v>
+      <c r="B4" s="23" t="n">
+        <v>46261</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1645,217 +1645,217 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Mes M+1 (Sep26-Sep26)</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
-        <v>63.76</v>
-      </c>
-      <c r="C6" s="28" t="n">
+      <c r="B6" s="25" t="n">
+        <v>65.89</v>
+      </c>
+      <c r="C6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Mes M+2 (Oct26-Oct26)</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
-        <v>64.68000000000001</v>
-      </c>
-      <c r="C7" s="28" t="n">
+      <c r="B7" s="25" t="n">
+        <v>64.98999999999999</v>
+      </c>
+      <c r="C7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Mes M+3 (Nov26-Nov26)</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
-        <v>64</v>
-      </c>
-      <c r="C8" s="28" t="n">
+      <c r="B8" s="25" t="n">
+        <v>66</v>
+      </c>
+      <c r="C8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+1 (Oct26-Dec26)</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
-        <v>63.95</v>
-      </c>
-      <c r="C9" s="28" t="n">
+      <c r="B9" s="25" t="n">
+        <v>65.63</v>
+      </c>
+      <c r="C9" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+2 (Jan27-Mar27)</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
-        <v>63.33</v>
-      </c>
-      <c r="C10" s="28" t="n">
+      <c r="B10" s="25" t="n">
+        <v>64.22</v>
+      </c>
+      <c r="C10" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+3 (Apr27-Jun27)</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
-        <v>44.41</v>
-      </c>
-      <c r="C11" s="28" t="n">
+      <c r="B11" s="25" t="n">
+        <v>45.21</v>
+      </c>
+      <c r="C11" s="26" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+4 (Jul27-Sep27)</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
-        <v>41.45</v>
-      </c>
-      <c r="C12" s="28" t="n">
+      <c r="B12" s="25" t="n">
+        <v>42.12</v>
+      </c>
+      <c r="C12" s="26" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Verano (abr-sep) (Apr27-Sep27)</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
-        <v>42.93</v>
-      </c>
-      <c r="C13" s="28" t="n">
+      <c r="B13" s="25" t="n">
+        <v>43.66</v>
+      </c>
+      <c r="C13" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Invierno (oct-mar) (Oct26-Mar27)</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="C14" s="28" t="n">
+      <c r="B14" s="25" t="n">
+        <v>65.58</v>
+      </c>
+      <c r="C14" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Año Y+1 (Jan27-Dec27)</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n">
-        <v>47.46</v>
-      </c>
-      <c r="C15" s="28" t="n">
+      <c r="B15" s="25" t="n">
+        <v>48.18</v>
+      </c>
+      <c r="C15" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Año Y+2 (Jan28-Dec28)</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
-        <v>31.81</v>
-      </c>
-      <c r="C16" s="28" t="n">
+      <c r="B16" s="25" t="n">
+        <v>31.97</v>
+      </c>
+      <c r="C16" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Suma de pesos (debe ser 12)</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="31">
         <f>SUM(C6:C16)</f>
         <v/>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="22">
         <f>IF(B18=12,"OK","⚠")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>FORWARD PRÓXIMOS 12 MESES (€/MWh)</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="33">
         <f>SUMPRODUCT(B6:B16,C6:C16)/SUM(C6:C16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Spot del mes en curso (€/MWh)</t>
         </is>
       </c>
-      <c r="B20" s="33">
-        <f>MIBGAS_Spot!E33</f>
+      <c r="B20" s="31">
+        <f>MIBGAS_Spot!E34</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>Contango/backwardation (forward − spot)</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="31">
         <f>B19-B20</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-29
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E34</f>
+        <f>E35</f>
         <v/>
       </c>
     </row>
@@ -1315,14 +1315,11 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E34" s="19">
-        <f>AVERAGE(E6:E33)</f>
-        <v/>
+      <c r="D34" s="13" t="n">
+        <v>46263</v>
+      </c>
+      <c r="E34" s="12" t="n">
+        <v>66.67</v>
       </c>
     </row>
     <row r="35">
@@ -1332,10 +1329,14 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D35" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E35" s="19">
+        <f>AVERAGE(E6:E34)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -1345,6 +1346,11 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
+      <c r="D36" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -1546,12 +1552,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D35:H35"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D36:H36"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1561,7 +1567,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E33">
+  <conditionalFormatting sqref="E6:E34">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1619,7 +1625,7 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1651,7 +1657,7 @@
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>65.89</v>
+        <v>68.69</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>1</v>
@@ -1669,7 +1675,7 @@
         </is>
       </c>
       <c r="B7" s="25" t="n">
-        <v>64.98999999999999</v>
+        <v>66.42</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>0</v>
@@ -1687,7 +1693,7 @@
         </is>
       </c>
       <c r="B8" s="25" t="n">
-        <v>66</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>0</v>
@@ -1705,7 +1711,7 @@
         </is>
       </c>
       <c r="B9" s="25" t="n">
-        <v>65.63</v>
+        <v>66</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>3</v>
@@ -1723,7 +1729,7 @@
         </is>
       </c>
       <c r="B10" s="25" t="n">
-        <v>64.22</v>
+        <v>62.85</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>3</v>
@@ -1741,7 +1747,7 @@
         </is>
       </c>
       <c r="B11" s="25" t="n">
-        <v>45.21</v>
+        <v>43.72</v>
       </c>
       <c r="C11" s="26" t="n">
         <v>3</v>
@@ -1754,7 +1760,7 @@
         </is>
       </c>
       <c r="B12" s="25" t="n">
-        <v>42.12</v>
+        <v>42.82</v>
       </c>
       <c r="C12" s="26" t="n">
         <v>2</v>
@@ -1767,7 +1773,7 @@
         </is>
       </c>
       <c r="B13" s="25" t="n">
-        <v>43.66</v>
+        <v>43.27</v>
       </c>
       <c r="C13" s="26" t="n">
         <v>0</v>
@@ -1780,7 +1786,7 @@
         </is>
       </c>
       <c r="B14" s="25" t="n">
-        <v>65.58</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="C14" s="26" t="n">
         <v>0</v>
@@ -1793,7 +1799,7 @@
         </is>
       </c>
       <c r="B15" s="25" t="n">
-        <v>48.18</v>
+        <v>47.83</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>0</v>
@@ -1806,7 +1812,7 @@
         </is>
       </c>
       <c r="B16" s="25" t="n">
-        <v>31.97</v>
+        <v>31.77</v>
       </c>
       <c r="C16" s="26" t="n">
         <v>0</v>
@@ -1845,7 +1851,7 @@
         </is>
       </c>
       <c r="B20" s="31">
-        <f>MIBGAS_Spot!E34</f>
+        <f>MIBGAS_Spot!E35</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-30
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E36</f>
+        <f>E37</f>
         <v/>
       </c>
     </row>
@@ -1335,10 +1335,10 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="18" t="n">
+      <c r="D35" s="13" t="n">
         <v>46264</v>
       </c>
-      <c r="E35" s="19" t="n">
+      <c r="E35" s="12" t="n">
         <v>66.7</v>
       </c>
     </row>
@@ -1349,14 +1349,11 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
-      <c r="D36" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E36" s="21">
-        <f>AVERAGE(E6:E35)</f>
-        <v/>
+      <c r="D36" s="18" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E36" s="19" t="n">
+        <v>67.11</v>
       </c>
     </row>
     <row r="37">
@@ -1366,10 +1363,14 @@
       <c r="B37" s="12" t="n">
         <v>32.58</v>
       </c>
-      <c r="D37" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D37" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E37" s="21">
+        <f>AVERAGE(E6:E36)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -1378,6 +1379,11 @@
       </c>
       <c r="B38" s="12" t="n">
         <v>31.84</v>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1568,7 +1574,7 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="D38:H38"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1579,7 +1585,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E35">
+  <conditionalFormatting sqref="E6:E36">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1863,7 +1869,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E36</f>
+        <f>MIBGAS_Spot!E37</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-31
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -203,12 +203,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1349,10 +1343,10 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
-      <c r="D36" s="18" t="n">
+      <c r="D36" s="13" t="n">
         <v>46265</v>
       </c>
-      <c r="E36" s="19" t="n">
+      <c r="E36" s="12" t="n">
         <v>67.11</v>
       </c>
     </row>
@@ -1363,12 +1357,12 @@
       <c r="B37" s="12" t="n">
         <v>32.58</v>
       </c>
-      <c r="D37" s="20" t="inlineStr">
+      <c r="D37" s="18" t="inlineStr">
         <is>
           <t>MEDIA MES</t>
         </is>
       </c>
-      <c r="E37" s="21">
+      <c r="E37" s="19">
         <f>AVERAGE(E6:E36)</f>
         <v/>
       </c>
@@ -1380,7 +1374,7 @@
       <c r="B38" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D38" s="22" t="inlineStr">
+      <c r="D38" s="20" t="inlineStr">
         <is>
           <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
         </is>
@@ -1470,103 +1464,103 @@
       <c r="A49" s="11" t="n">
         <v>46235</v>
       </c>
-      <c r="B49" s="23" t="n"/>
+      <c r="B49" s="21" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n">
         <v>46266</v>
       </c>
-      <c r="B50" s="23" t="n"/>
+      <c r="B50" s="21" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="B51" s="23" t="n"/>
+      <c r="B51" s="21" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
         <v>46327</v>
       </c>
-      <c r="B52" s="23" t="n"/>
+      <c r="B52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
         <v>46357</v>
       </c>
-      <c r="B53" s="23" t="n"/>
+      <c r="B53" s="21" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
         <v>46388</v>
       </c>
-      <c r="B54" s="23" t="n"/>
+      <c r="B54" s="21" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
         <v>46419</v>
       </c>
-      <c r="B55" s="23" t="n"/>
+      <c r="B55" s="21" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
         <v>46447</v>
       </c>
-      <c r="B56" s="23" t="n"/>
+      <c r="B56" s="21" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
         <v>46478</v>
       </c>
-      <c r="B57" s="23" t="n"/>
+      <c r="B57" s="21" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
         <v>46508</v>
       </c>
-      <c r="B58" s="23" t="n"/>
+      <c r="B58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
         <v>46539</v>
       </c>
-      <c r="B59" s="23" t="n"/>
+      <c r="B59" s="21" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
         <v>46569</v>
       </c>
-      <c r="B60" s="23" t="n"/>
+      <c r="B60" s="21" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
         <v>46600</v>
       </c>
-      <c r="B61" s="23" t="n"/>
+      <c r="B61" s="21" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
         <v>46631</v>
       </c>
-      <c r="B62" s="23" t="n"/>
+      <c r="B62" s="21" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
         <v>46661</v>
       </c>
-      <c r="B63" s="23" t="n"/>
+      <c r="B63" s="21" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
         <v>46692</v>
       </c>
-      <c r="B64" s="23" t="n"/>
+      <c r="B64" s="21" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
         <v>46722</v>
       </c>
-      <c r="B65" s="23" t="n"/>
+      <c r="B65" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1637,13 +1631,13 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Fecha de la curva:</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
-        <v>46262</v>
+      <c r="B4" s="23" t="n">
+        <v>46265</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1669,217 +1663,217 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Mes M+1 (Sep26-Sep26)</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
-        <v>68.69</v>
-      </c>
-      <c r="C6" s="28" t="n">
+      <c r="B6" s="25" t="n">
+        <v>70.08</v>
+      </c>
+      <c r="C6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Mes M+2 (Oct26-Oct26)</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
-        <v>66.42</v>
-      </c>
-      <c r="C7" s="28" t="n">
+      <c r="B7" s="25" t="n">
+        <v>69.17</v>
+      </c>
+      <c r="C7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Mes M+3 (Nov26-Nov26)</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
-        <v>65.40000000000001</v>
-      </c>
-      <c r="C8" s="28" t="n">
+      <c r="B8" s="25" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="C8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+1 (Oct26-Dec26)</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
-        <v>66</v>
-      </c>
-      <c r="C9" s="28" t="n">
+      <c r="B9" s="25" t="n">
+        <v>68.88</v>
+      </c>
+      <c r="C9" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+2 (Jan27-Mar27)</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
-        <v>62.85</v>
-      </c>
-      <c r="C10" s="28" t="n">
+      <c r="B10" s="25" t="n">
+        <v>66.34999999999999</v>
+      </c>
+      <c r="C10" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+3 (Apr27-Jun27)</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
-        <v>43.72</v>
-      </c>
-      <c r="C11" s="28" t="n">
+      <c r="B11" s="25" t="n">
+        <v>47.41</v>
+      </c>
+      <c r="C11" s="26" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+4 (Jul27-Sep27)</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
-        <v>42.82</v>
-      </c>
-      <c r="C12" s="28" t="n">
+      <c r="B12" s="25" t="n">
+        <v>44.35</v>
+      </c>
+      <c r="C12" s="26" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Verano (abr-sep) (Apr27-Sep27)</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
-        <v>43.27</v>
-      </c>
-      <c r="C13" s="28" t="n">
+      <c r="B13" s="25" t="n">
+        <v>45.87</v>
+      </c>
+      <c r="C13" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Invierno (oct-mar) (Oct26-Mar27)</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n">
-        <v>64.18000000000001</v>
-      </c>
-      <c r="C14" s="28" t="n">
+      <c r="B14" s="25" t="n">
+        <v>67.63</v>
+      </c>
+      <c r="C14" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Año Y+1 (Jan27-Dec27)</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n">
-        <v>47.83</v>
-      </c>
-      <c r="C15" s="28" t="n">
+      <c r="B15" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="C15" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Año Y+2 (Jan28-Dec28)</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
-        <v>31.77</v>
-      </c>
-      <c r="C16" s="28" t="n">
+      <c r="B16" s="25" t="n">
+        <v>33.19</v>
+      </c>
+      <c r="C16" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Suma de pesos (debe ser 12)</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="31">
         <f>SUM(C6:C16)</f>
         <v/>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="22">
         <f>IF(B18=12,"OK","⚠")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>FORWARD PRÓXIMOS 12 MESES (€/MWh)</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="33">
         <f>SUMPRODUCT(B6:B16,C6:C16)/SUM(C6:C16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Spot del mes en curso (€/MWh)</t>
         </is>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="31">
         <f>MIBGAS_Spot!E37</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>Contango/backwardation (forward − spot)</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="31">
         <f>B19-B20</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-01
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -199,10 +199,10 @@
     <xf numFmtId="168" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -210,6 +210,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -770,7 +776,7 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>MES EN CURSO (Aug-2026)</t>
+          <t>MES EN CURSO (Sep-2026)</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
@@ -819,10 +825,10 @@
         <v>60.62</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>59.16</v>
+        <v>70.27</v>
       </c>
       <c r="J6" s="14">
         <f>A42</f>
@@ -840,11 +846,11 @@
       <c r="B7" s="12" t="n">
         <v>52.17</v>
       </c>
-      <c r="D7" s="13" t="n">
-        <v>46236</v>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>60.75</v>
+      <c r="D7" s="16" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>72.48</v>
       </c>
       <c r="J7" s="14">
         <f>A43</f>
@@ -862,11 +868,14 @@
       <c r="B8" s="12" t="n">
         <v>43.67</v>
       </c>
-      <c r="D8" s="13" t="n">
-        <v>46237</v>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>58.66</v>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E8" s="19">
+        <f>AVERAGE(E6:E7)</f>
+        <v/>
       </c>
       <c r="J8" s="14">
         <f>A44</f>
@@ -884,11 +893,10 @@
       <c r="B9" s="12" t="n">
         <v>38.09</v>
       </c>
-      <c r="D9" s="13" t="n">
-        <v>46238</v>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>57.82</v>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
       <c r="J9" s="14">
         <f>A45</f>
@@ -906,12 +914,6 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
-      <c r="D10" s="13" t="n">
-        <v>46239</v>
-      </c>
-      <c r="E10" s="12" t="n">
-        <v>56.1</v>
-      </c>
       <c r="J10" s="14">
         <f>A46</f>
         <v/>
@@ -928,12 +930,6 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
-      <c r="D11" s="13" t="n">
-        <v>46240</v>
-      </c>
-      <c r="E11" s="12" t="n">
-        <v>52.41</v>
-      </c>
       <c r="J11" s="14">
         <f>A47</f>
         <v/>
@@ -950,12 +946,6 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
-      <c r="D12" s="13" t="n">
-        <v>46241</v>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>55.84</v>
-      </c>
       <c r="J12" s="14">
         <f>A48</f>
         <v/>
@@ -972,12 +962,6 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
-      <c r="D13" s="13" t="n">
-        <v>46242</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>54.9</v>
-      </c>
       <c r="J13" s="14">
         <f>A49</f>
         <v/>
@@ -994,12 +978,6 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
-      <c r="D14" s="13" t="n">
-        <v>46243</v>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>55.95</v>
-      </c>
       <c r="J14" s="14">
         <f>A50</f>
         <v/>
@@ -1016,12 +994,6 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
-      <c r="D15" s="13" t="n">
-        <v>46244</v>
-      </c>
-      <c r="E15" s="12" t="n">
-        <v>56.62</v>
-      </c>
       <c r="J15" s="14">
         <f>A51</f>
         <v/>
@@ -1038,12 +1010,6 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="13" t="n">
-        <v>46245</v>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>60.44</v>
-      </c>
       <c r="J16" s="14">
         <f>A52</f>
         <v/>
@@ -1060,12 +1026,6 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="13" t="n">
-        <v>46246</v>
-      </c>
-      <c r="E17" s="12" t="n">
-        <v>59.05</v>
-      </c>
       <c r="J17" s="14">
         <f>A53</f>
         <v/>
@@ -1082,19 +1042,13 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="13" t="n">
-        <v>46247</v>
-      </c>
-      <c r="E18" s="12" t="n">
-        <v>60.45</v>
-      </c>
-      <c r="J18" s="16" t="inlineStr">
-        <is>
-          <t>Aug</t>
-        </is>
-      </c>
-      <c r="K18" s="17">
-        <f>E37</f>
+      <c r="J18" s="21" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K18" s="22">
+        <f>E8</f>
         <v/>
       </c>
     </row>
@@ -1105,12 +1059,6 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="13" t="n">
-        <v>46248</v>
-      </c>
-      <c r="E19" s="12" t="n">
-        <v>60.77</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="n">
@@ -1119,12 +1067,6 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="13" t="n">
-        <v>46249</v>
-      </c>
-      <c r="E20" s="12" t="n">
-        <v>60.81</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -1133,12 +1075,6 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="13" t="n">
-        <v>46250</v>
-      </c>
-      <c r="E21" s="12" t="n">
-        <v>62.41</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
@@ -1147,12 +1083,6 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="13" t="n">
-        <v>46251</v>
-      </c>
-      <c r="E22" s="12" t="n">
-        <v>63.46</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
@@ -1161,12 +1091,6 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="13" t="n">
-        <v>46252</v>
-      </c>
-      <c r="E23" s="12" t="n">
-        <v>61.77</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n">
@@ -1175,12 +1099,6 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="13" t="n">
-        <v>46253</v>
-      </c>
-      <c r="E24" s="12" t="n">
-        <v>63.61</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">
@@ -1189,12 +1107,6 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="13" t="n">
-        <v>46254</v>
-      </c>
-      <c r="E25" s="12" t="n">
-        <v>63.47</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1203,12 +1115,6 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="13" t="n">
-        <v>46255</v>
-      </c>
-      <c r="E26" s="12" t="n">
-        <v>65.61</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1217,12 +1123,6 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="13" t="n">
-        <v>46256</v>
-      </c>
-      <c r="E27" s="12" t="n">
-        <v>66.31</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
@@ -1231,12 +1131,6 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="13" t="n">
-        <v>46257</v>
-      </c>
-      <c r="E28" s="12" t="n">
-        <v>66.68000000000001</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n">
@@ -1245,12 +1139,6 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="13" t="n">
-        <v>46258</v>
-      </c>
-      <c r="E29" s="12" t="n">
-        <v>66.22</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
@@ -1259,12 +1147,6 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
-      <c r="D30" s="13" t="n">
-        <v>46259</v>
-      </c>
-      <c r="E30" s="12" t="n">
-        <v>67.97</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
@@ -1273,12 +1155,6 @@
       <c r="B31" s="12" t="n">
         <v>50.4</v>
       </c>
-      <c r="D31" s="13" t="n">
-        <v>46260</v>
-      </c>
-      <c r="E31" s="12" t="n">
-        <v>66.09999999999999</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1287,12 +1163,6 @@
       <c r="B32" s="12" t="n">
         <v>41.41</v>
       </c>
-      <c r="D32" s="13" t="n">
-        <v>46261</v>
-      </c>
-      <c r="E32" s="12" t="n">
-        <v>65.86</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n">
@@ -1301,12 +1171,6 @@
       <c r="B33" s="12" t="n">
         <v>33.76</v>
       </c>
-      <c r="D33" s="13" t="n">
-        <v>46262</v>
-      </c>
-      <c r="E33" s="12" t="n">
-        <v>68.38</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
@@ -1315,12 +1179,6 @@
       <c r="B34" s="12" t="n">
         <v>34.02</v>
       </c>
-      <c r="D34" s="13" t="n">
-        <v>46263</v>
-      </c>
-      <c r="E34" s="12" t="n">
-        <v>66.67</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n">
@@ -1329,12 +1187,6 @@
       <c r="B35" s="12" t="n">
         <v>36.67</v>
       </c>
-      <c r="D35" s="13" t="n">
-        <v>46264</v>
-      </c>
-      <c r="E35" s="12" t="n">
-        <v>66.7</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -1343,12 +1195,6 @@
       <c r="B36" s="12" t="n">
         <v>33.94</v>
       </c>
-      <c r="D36" s="13" t="n">
-        <v>46265</v>
-      </c>
-      <c r="E36" s="12" t="n">
-        <v>67.11</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -1357,15 +1203,6 @@
       <c r="B37" s="12" t="n">
         <v>32.58</v>
       </c>
-      <c r="D37" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E37" s="19">
-        <f>AVERAGE(E6:E36)</f>
-        <v/>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
@@ -1374,11 +1211,6 @@
       <c r="B38" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D38" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n">
@@ -1464,103 +1296,105 @@
       <c r="A49" s="11" t="n">
         <v>46235</v>
       </c>
-      <c r="B49" s="21" t="n"/>
+      <c r="B49" s="12" t="n">
+        <v>61.87</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n">
         <v>46266</v>
       </c>
-      <c r="B50" s="21" t="n"/>
+      <c r="B50" s="23" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="B51" s="21" t="n"/>
+      <c r="B51" s="23" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
         <v>46327</v>
       </c>
-      <c r="B52" s="21" t="n"/>
+      <c r="B52" s="23" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
         <v>46357</v>
       </c>
-      <c r="B53" s="21" t="n"/>
+      <c r="B53" s="23" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
         <v>46388</v>
       </c>
-      <c r="B54" s="21" t="n"/>
+      <c r="B54" s="23" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
         <v>46419</v>
       </c>
-      <c r="B55" s="21" t="n"/>
+      <c r="B55" s="23" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
         <v>46447</v>
       </c>
-      <c r="B56" s="21" t="n"/>
+      <c r="B56" s="23" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
         <v>46478</v>
       </c>
-      <c r="B57" s="21" t="n"/>
+      <c r="B57" s="23" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
         <v>46508</v>
       </c>
-      <c r="B58" s="21" t="n"/>
+      <c r="B58" s="23" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
         <v>46539</v>
       </c>
-      <c r="B59" s="21" t="n"/>
+      <c r="B59" s="23" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
         <v>46569</v>
       </c>
-      <c r="B60" s="21" t="n"/>
+      <c r="B60" s="23" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
         <v>46600</v>
       </c>
-      <c r="B61" s="21" t="n"/>
+      <c r="B61" s="23" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
         <v>46631</v>
       </c>
-      <c r="B62" s="21" t="n"/>
+      <c r="B62" s="23" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
         <v>46661</v>
       </c>
-      <c r="B63" s="21" t="n"/>
+      <c r="B63" s="23" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
         <v>46692</v>
       </c>
-      <c r="B64" s="21" t="n"/>
+      <c r="B64" s="23" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
         <v>46722</v>
       </c>
-      <c r="B65" s="21" t="n"/>
+      <c r="B65" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1568,8 +1402,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D38:H38"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D9:H9"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1579,7 +1413,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E36">
+  <conditionalFormatting sqref="E6:E7">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1631,13 +1465,13 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Fecha de la curva:</t>
         </is>
       </c>
-      <c r="B4" s="23" t="n">
-        <v>46265</v>
+      <c r="B4" s="25" t="n">
+        <v>46266</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1663,217 +1497,217 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>Mes M+1 (Sep26-Sep26)</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="n">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Mes M+1 (Oct26-Oct26)</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="n">
         <v>70.08</v>
       </c>
-      <c r="C6" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="27" t="inlineStr">
+      <c r="C6" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>Mes M+2 (Oct26-Oct26)</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="n">
-        <v>69.17</v>
-      </c>
-      <c r="C7" s="26" t="n">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Mes M+2 (Nov26-Nov26)</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>70.38</v>
+      </c>
+      <c r="C7" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>Mes M+3 (Nov26-Nov26)</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="n">
-        <v>68.89</v>
-      </c>
-      <c r="C8" s="26" t="n">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Mes M+3 (Dec26-Dec26)</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>70.65000000000001</v>
+      </c>
+      <c r="C8" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="27" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Trimestre Q+1 (Oct26-Dec26)</t>
         </is>
       </c>
-      <c r="B9" s="25" t="n">
-        <v>68.88</v>
-      </c>
-      <c r="C9" s="26" t="n">
+      <c r="B9" s="27" t="n">
+        <v>69.95</v>
+      </c>
+      <c r="C9" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="27" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>Trimestre Q+2 (Jan27-Mar27)</t>
         </is>
       </c>
-      <c r="B10" s="25" t="n">
-        <v>66.34999999999999</v>
-      </c>
-      <c r="C10" s="26" t="n">
+      <c r="B10" s="27" t="n">
+        <v>68.34999999999999</v>
+      </c>
+      <c r="C10" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="27" t="inlineStr">
+      <c r="E10" s="29" t="inlineStr">
         <is>
           <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Trimestre Q+3 (Apr27-Jun27)</t>
         </is>
       </c>
-      <c r="B11" s="25" t="n">
-        <v>47.41</v>
-      </c>
-      <c r="C11" s="26" t="n">
+      <c r="B11" s="27" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="C11" s="28" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>Trimestre Q+4 (Jul27-Sep27)</t>
         </is>
       </c>
-      <c r="B12" s="25" t="n">
-        <v>44.35</v>
-      </c>
-      <c r="C12" s="26" t="n">
-        <v>2</v>
+      <c r="B12" s="27" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="C12" s="28" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Verano (abr-sep) (Apr27-Sep27)</t>
         </is>
       </c>
-      <c r="B13" s="25" t="n">
-        <v>45.87</v>
-      </c>
-      <c r="C13" s="26" t="n">
+      <c r="B13" s="27" t="n">
+        <v>46.81</v>
+      </c>
+      <c r="C13" s="28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Invierno (oct-mar) (Oct26-Mar27)</t>
         </is>
       </c>
-      <c r="B14" s="25" t="n">
-        <v>67.63</v>
-      </c>
-      <c r="C14" s="26" t="n">
+      <c r="B14" s="27" t="n">
+        <v>69</v>
+      </c>
+      <c r="C14" s="28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>Año Y+1 (Jan27-Dec27)</t>
         </is>
       </c>
-      <c r="B15" s="25" t="n">
-        <v>50</v>
-      </c>
-      <c r="C15" s="26" t="n">
+      <c r="B15" s="27" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="C15" s="28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Año Y+2 (Jan28-Dec28)</t>
         </is>
       </c>
-      <c r="B16" s="25" t="n">
-        <v>33.19</v>
-      </c>
-      <c r="C16" s="26" t="n">
+      <c r="B16" s="27" t="n">
+        <v>33.76</v>
+      </c>
+      <c r="C16" s="28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>Suma de pesos (debe ser 12)</t>
         </is>
       </c>
-      <c r="B18" s="31">
+      <c r="B18" s="33">
         <f>SUM(C6:C16)</f>
         <v/>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="24">
         <f>IF(B18=12,"OK","⚠")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" s="34" t="inlineStr">
         <is>
           <t>FORWARD PRÓXIMOS 12 MESES (€/MWh)</t>
         </is>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="35">
         <f>SUMPRODUCT(B6:B16,C6:C16)/SUM(C6:C16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t>Spot del mes en curso (€/MWh)</t>
         </is>
       </c>
-      <c r="B20" s="31">
-        <f>MIBGAS_Spot!E37</f>
+      <c r="B20" s="33">
+        <f>MIBGAS_Spot!E8</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="30" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>Contango/backwardation (forward − spot)</t>
         </is>
       </c>
-      <c r="B21" s="31">
+      <c r="B21" s="33">
         <f>B19-B20</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-02
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -846,10 +846,10 @@
       <c r="B7" s="12" t="n">
         <v>52.17</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="13" t="n">
         <v>46267</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="12" t="n">
         <v>72.48</v>
       </c>
       <c r="J7" s="14">
@@ -868,14 +868,11 @@
       <c r="B8" s="12" t="n">
         <v>43.67</v>
       </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E8" s="19">
-        <f>AVERAGE(E6:E7)</f>
-        <v/>
+      <c r="D8" s="16" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>73.91</v>
       </c>
       <c r="J8" s="14">
         <f>A44</f>
@@ -893,10 +890,14 @@
       <c r="B9" s="12" t="n">
         <v>38.09</v>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E9" s="19">
+        <f>AVERAGE(E6:E8)</f>
+        <v/>
       </c>
       <c r="J9" s="14">
         <f>A45</f>
@@ -914,6 +915,11 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J10" s="14">
         <f>A46</f>
         <v/>
@@ -1048,7 +1054,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E8</f>
+        <f>E9</f>
         <v/>
       </c>
     </row>
@@ -1400,10 +1406,10 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D10:H10"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D9:H9"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1413,7 +1419,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E7">
+  <conditionalFormatting sqref="E6:E8">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1471,7 +1477,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1503,7 +1509,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>70.08</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1521,7 +1527,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>70.38</v>
+        <v>72.7</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1539,7 +1545,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>70.65000000000001</v>
+        <v>72.94</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1557,7 +1563,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>69.95</v>
+        <v>72.58</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1575,7 +1581,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>68.34999999999999</v>
+        <v>69.44</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1593,7 +1599,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>48.2</v>
+        <v>50.36</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1606,7 +1612,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>45.2</v>
+        <v>47.1</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1619,7 +1625,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>46.81</v>
+        <v>48.72</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1632,7 +1638,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>69</v>
+        <v>70.88</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1645,7 +1651,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>51.6</v>
+        <v>52.6</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1658,7 +1664,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>33.76</v>
+        <v>34.99</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1697,7 +1703,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E8</f>
+        <f>MIBGAS_Spot!E9</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-03
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -868,10 +868,10 @@
       <c r="B8" s="12" t="n">
         <v>43.67</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="13" t="n">
         <v>46268</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="12" t="n">
         <v>73.91</v>
       </c>
       <c r="J8" s="14">
@@ -890,14 +890,11 @@
       <c r="B9" s="12" t="n">
         <v>38.09</v>
       </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E9" s="19">
-        <f>AVERAGE(E6:E8)</f>
-        <v/>
+      <c r="D9" s="16" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>72.09999999999999</v>
       </c>
       <c r="J9" s="14">
         <f>A45</f>
@@ -915,10 +912,14 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E10" s="19">
+        <f>AVERAGE(E6:E9)</f>
+        <v/>
       </c>
       <c r="J10" s="14">
         <f>A46</f>
@@ -936,6 +937,11 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J11" s="14">
         <f>A47</f>
         <v/>
@@ -1054,7 +1060,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E9</f>
+        <f>E10</f>
         <v/>
       </c>
     </row>
@@ -1406,8 +1412,8 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D10:H10"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D11:H11"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1419,7 +1425,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E8">
+  <conditionalFormatting sqref="E6:E9">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1477,7 +1483,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1509,7 +1515,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>72.65000000000001</v>
+        <v>71.81</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1527,7 +1533,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>72.7</v>
+        <v>71.55</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1545,7 +1551,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>72.94</v>
+        <v>70.65000000000001</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1563,7 +1569,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>72.58</v>
+        <v>70.84</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1581,7 +1587,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>69.44</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1599,7 +1605,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>50.36</v>
+        <v>49.27</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1612,7 +1618,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>47.1</v>
+        <v>46.13</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1625,7 +1631,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>48.72</v>
+        <v>47.69</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1638,7 +1644,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>70.88</v>
+        <v>69.08</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1651,7 +1657,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>52.6</v>
+        <v>52.08</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1664,7 +1670,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>34.99</v>
+        <v>34.23</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1703,7 +1709,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E9</f>
+        <f>MIBGAS_Spot!E10</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-04
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -890,10 +890,10 @@
       <c r="B9" s="12" t="n">
         <v>38.09</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="13" t="n">
         <v>46269</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="12" t="n">
         <v>72.09999999999999</v>
       </c>
       <c r="J9" s="14">
@@ -912,14 +912,11 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E10" s="19">
-        <f>AVERAGE(E6:E9)</f>
-        <v/>
+      <c r="D10" s="16" t="n">
+        <v>46270</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>72.84999999999999</v>
       </c>
       <c r="J10" s="14">
         <f>A46</f>
@@ -937,10 +934,14 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E11" s="19">
+        <f>AVERAGE(E6:E10)</f>
+        <v/>
       </c>
       <c r="J11" s="14">
         <f>A47</f>
@@ -958,6 +959,11 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J12" s="14">
         <f>A48</f>
         <v/>
@@ -1060,7 +1066,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E10</f>
+        <f>E11</f>
         <v/>
       </c>
     </row>
@@ -1410,10 +1416,10 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D12:H12"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D11:H11"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1425,7 +1431,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E9">
+  <conditionalFormatting sqref="E6:E10">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1483,7 +1489,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1515,7 +1521,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>71.81</v>
+        <v>70.53</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1533,7 +1539,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>71.55</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1551,7 +1557,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>70.65000000000001</v>
+        <v>70.25</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1569,7 +1575,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>70.84</v>
+        <v>70.7</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1587,7 +1593,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>68.90000000000001</v>
+        <v>66.92</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1605,7 +1611,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>49.27</v>
+        <v>50.07</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1618,7 +1624,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>46.13</v>
+        <v>46.73</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1631,7 +1637,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>47.69</v>
+        <v>48.39</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1657,7 +1663,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>52.08</v>
+        <v>52.43</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1670,7 +1676,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>34.23</v>
+        <v>34.58</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1709,7 +1715,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E10</f>
+        <f>MIBGAS_Spot!E11</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-05
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -912,10 +912,10 @@
       <c r="B10" s="12" t="n">
         <v>29.23</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="13" t="n">
         <v>46270</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="12" t="n">
         <v>72.84999999999999</v>
       </c>
       <c r="J10" s="14">
@@ -934,14 +934,11 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E11" s="19">
-        <f>AVERAGE(E6:E10)</f>
-        <v/>
+      <c r="D11" s="16" t="n">
+        <v>46271</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>79.03</v>
       </c>
       <c r="J11" s="14">
         <f>A47</f>
@@ -959,10 +956,14 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E12" s="19">
+        <f>AVERAGE(E6:E11)</f>
+        <v/>
       </c>
       <c r="J12" s="14">
         <f>A48</f>
@@ -980,6 +981,11 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J13" s="14">
         <f>A49</f>
         <v/>
@@ -1066,7 +1072,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E11</f>
+        <f>E12</f>
         <v/>
       </c>
     </row>
@@ -1416,10 +1422,10 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D12:H12"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D13:H13"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1431,7 +1437,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E10">
+  <conditionalFormatting sqref="E6:E11">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1715,7 +1721,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E11</f>
+        <f>MIBGAS_Spot!E12</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-06
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -934,10 +934,10 @@
       <c r="B11" s="12" t="n">
         <v>30.93</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="13" t="n">
         <v>46271</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="12" t="n">
         <v>79.03</v>
       </c>
       <c r="J11" s="14">
@@ -956,14 +956,11 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E12" s="19">
-        <f>AVERAGE(E6:E11)</f>
-        <v/>
+      <c r="D12" s="16" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>77.63</v>
       </c>
       <c r="J12" s="14">
         <f>A48</f>
@@ -981,10 +978,14 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E13" s="19">
+        <f>AVERAGE(E6:E12)</f>
+        <v/>
       </c>
       <c r="J13" s="14">
         <f>A49</f>
@@ -1002,6 +1003,11 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J14" s="14">
         <f>A50</f>
         <v/>
@@ -1072,7 +1078,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E12</f>
+        <f>E13</f>
         <v/>
       </c>
     </row>
@@ -1425,9 +1431,9 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D13:H13"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D14:H14"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1437,7 +1443,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E11">
+  <conditionalFormatting sqref="E6:E12">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1721,7 +1727,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E12</f>
+        <f>MIBGAS_Spot!E13</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-07
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -956,10 +956,10 @@
       <c r="B12" s="12" t="n">
         <v>30.55</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="13" t="n">
         <v>46272</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="12" t="n">
         <v>77.63</v>
       </c>
       <c r="J12" s="14">
@@ -978,14 +978,11 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E13" s="19">
-        <f>AVERAGE(E6:E12)</f>
-        <v/>
+      <c r="D13" s="16" t="n">
+        <v>46273</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>74.76000000000001</v>
       </c>
       <c r="J13" s="14">
         <f>A49</f>
@@ -1003,10 +1000,14 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E14" s="19">
+        <f>AVERAGE(E6:E13)</f>
+        <v/>
       </c>
       <c r="J14" s="14">
         <f>A50</f>
@@ -1024,6 +1025,11 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J15" s="14">
         <f>A51</f>
         <v/>
@@ -1078,7 +1084,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E13</f>
+        <f>E14</f>
         <v/>
       </c>
     </row>
@@ -1429,11 +1435,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D15:H15"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D14:H14"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1443,7 +1449,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E12">
+  <conditionalFormatting sqref="E6:E13">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1501,7 +1507,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1533,7 +1539,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>70.53</v>
+        <v>72.84</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1551,7 +1557,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>70.15000000000001</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1569,7 +1575,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>70.25</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1587,7 +1593,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>70.7</v>
+        <v>72.55</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1605,7 +1611,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>66.92</v>
+        <v>70.09</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1623,7 +1629,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>50.07</v>
+        <v>50.54</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1636,7 +1642,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>46.73</v>
+        <v>47.09</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1649,7 +1655,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>48.39</v>
+        <v>48.81</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1662,7 +1668,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>69.08</v>
+        <v>71.18000000000001</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1675,7 +1681,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>52.43</v>
+        <v>53.6</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1688,7 +1694,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>34.58</v>
+        <v>34.49</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1727,7 +1733,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E13</f>
+        <f>MIBGAS_Spot!E14</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-08
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -978,10 +978,10 @@
       <c r="B13" s="12" t="n">
         <v>33.86</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="13" t="n">
         <v>46273</v>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="12" t="n">
         <v>74.76000000000001</v>
       </c>
       <c r="J13" s="14">
@@ -1000,14 +1000,11 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E14" s="19">
-        <f>AVERAGE(E6:E13)</f>
-        <v/>
+      <c r="D14" s="16" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>77.44</v>
       </c>
       <c r="J14" s="14">
         <f>A50</f>
@@ -1025,10 +1022,14 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E15" s="19">
+        <f>AVERAGE(E6:E14)</f>
+        <v/>
       </c>
       <c r="J15" s="14">
         <f>A51</f>
@@ -1046,6 +1047,11 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J16" s="14">
         <f>A52</f>
         <v/>
@@ -1084,7 +1090,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E14</f>
+        <f>E15</f>
         <v/>
       </c>
     </row>
@@ -1435,8 +1441,8 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D15:H15"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D16:H16"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
@@ -1449,7 +1455,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E13">
+  <conditionalFormatting sqref="E6:E14">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1507,7 +1513,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1539,7 +1545,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>72.84</v>
+        <v>74.58</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1557,7 +1563,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>71.84999999999999</v>
+        <v>74.77</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1575,7 +1581,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>71.90000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1593,7 +1599,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>72.55</v>
+        <v>75.3</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1611,7 +1617,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>70.09</v>
+        <v>72.84</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1629,7 +1635,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>50.54</v>
+        <v>52.49</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1642,7 +1648,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>47.09</v>
+        <v>48.8</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1655,7 +1661,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>48.81</v>
+        <v>50.63</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1668,7 +1674,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>71.18000000000001</v>
+        <v>74.08</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1681,7 +1687,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>53.6</v>
+        <v>55.5</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1694,7 +1700,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>34.49</v>
+        <v>35.01</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1733,7 +1739,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E14</f>
+        <f>MIBGAS_Spot!E15</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-09
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1000,10 +1000,10 @@
       <c r="B14" s="12" t="n">
         <v>36.93</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="13" t="n">
         <v>46274</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="12" t="n">
         <v>77.44</v>
       </c>
       <c r="J14" s="14">
@@ -1022,14 +1022,11 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E15" s="19">
-        <f>AVERAGE(E6:E14)</f>
-        <v/>
+      <c r="D15" s="16" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>80.77</v>
       </c>
       <c r="J15" s="14">
         <f>A51</f>
@@ -1047,10 +1044,14 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E16" s="19">
+        <f>AVERAGE(E6:E15)</f>
+        <v/>
       </c>
       <c r="J16" s="14">
         <f>A52</f>
@@ -1068,6 +1069,11 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J17" s="14">
         <f>A53</f>
         <v/>
@@ -1090,7 +1096,7 @@
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E15</f>
+        <f>E16</f>
         <v/>
       </c>
     </row>
@@ -1442,10 +1448,10 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D16:H16"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D17:H17"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1455,7 +1461,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E14">
+  <conditionalFormatting sqref="E6:E15">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1513,7 +1519,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1545,7 +1551,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>74.58</v>
+        <v>78.18000000000001</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1563,7 +1569,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>74.77</v>
+        <v>77.89</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1581,7 +1587,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>74.2</v>
+        <v>77.98</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1599,7 +1605,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>75.3</v>
+        <v>78.31</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1617,7 +1623,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>72.84</v>
+        <v>75.37</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1635,7 +1641,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>52.49</v>
+        <v>54.48</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1648,7 +1654,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>48.8</v>
+        <v>50.38</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1661,7 +1667,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>50.63</v>
+        <v>52.42</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1674,7 +1680,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>74.08</v>
+        <v>76.98</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1687,7 +1693,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>55.5</v>
+        <v>57.15</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1700,7 +1706,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>35.01</v>
+        <v>35.59</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1739,7 +1745,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E15</f>
+        <f>MIBGAS_Spot!E16</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-10
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1022,10 +1022,10 @@
       <c r="B15" s="12" t="n">
         <v>43.11</v>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="13" t="n">
         <v>46275</v>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="12" t="n">
         <v>80.77</v>
       </c>
       <c r="J15" s="14">
@@ -1044,14 +1044,11 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E16" s="19">
-        <f>AVERAGE(E6:E15)</f>
-        <v/>
+      <c r="D16" s="16" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>83.45999999999999</v>
       </c>
       <c r="J16" s="14">
         <f>A52</f>
@@ -1069,10 +1066,14 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E17" s="19">
+        <f>AVERAGE(E6:E16)</f>
+        <v/>
       </c>
       <c r="J17" s="14">
         <f>A53</f>
@@ -1090,13 +1091,18 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J18" s="21" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
       <c r="K18" s="22">
-        <f>E16</f>
+        <f>E17</f>
         <v/>
       </c>
     </row>
@@ -1451,7 +1457,7 @@
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1461,7 +1467,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E15">
+  <conditionalFormatting sqref="E6:E16">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1519,7 +1525,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1551,7 +1557,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>78.18000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1569,7 +1575,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>77.89</v>
+        <v>80.15000000000001</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1587,7 +1593,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>77.98</v>
+        <v>79.69</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1605,7 +1611,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>78.31</v>
+        <v>80.39</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1623,7 +1629,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>75.37</v>
+        <v>77.68000000000001</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1641,7 +1647,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>54.48</v>
+        <v>57.09</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1654,7 +1660,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>50.38</v>
+        <v>52.45</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1667,7 +1673,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>52.42</v>
+        <v>54.75</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1680,7 +1686,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>76.98</v>
+        <v>79.63</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1693,7 +1699,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>57.15</v>
+        <v>59.63</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1706,7 +1712,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>35.59</v>
+        <v>36.89</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1745,7 +1751,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E16</f>
+        <f>MIBGAS_Spot!E17</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-09-11
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -209,13 +209,13 @@
     <xf numFmtId="4" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1044,10 +1044,10 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="16" t="n">
+      <c r="D16" s="13" t="n">
         <v>46276</v>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="12" t="n">
         <v>83.45999999999999</v>
       </c>
       <c r="J16" s="14">
@@ -1066,14 +1066,11 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E17" s="19">
-        <f>AVERAGE(E6:E16)</f>
-        <v/>
+      <c r="D17" s="16" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>81.36</v>
       </c>
       <c r="J17" s="14">
         <f>A53</f>
@@ -1091,18 +1088,22 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
-      </c>
-      <c r="J18" s="21" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E18" s="19">
+        <f>AVERAGE(E6:E17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="20" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="K18" s="22">
-        <f>E17</f>
+      <c r="K18" s="21">
+        <f>E18</f>
         <v/>
       </c>
     </row>
@@ -1112,6 +1113,11 @@
       </c>
       <c r="B19" s="12" t="n">
         <v>25.5</v>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1455,9 +1461,9 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D19:H19"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D18:H18"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1467,7 +1473,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E16">
+  <conditionalFormatting sqref="E6:E17">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1525,7 +1531,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1557,7 +1563,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>80.7</v>
+        <v>79.97</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>0</v>
@@ -1575,7 +1581,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>80.15000000000001</v>
+        <v>79.64</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1593,7 +1599,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>79.69</v>
+        <v>79.65000000000001</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1611,7 +1617,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>80.39</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1629,7 +1635,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>77.68000000000001</v>
+        <v>77.58</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1647,7 +1653,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>57.09</v>
+        <v>56.07</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1660,7 +1666,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>52.45</v>
+        <v>51.44</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>3</v>
@@ -1673,7 +1679,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>54.75</v>
+        <v>53.74</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1686,7 +1692,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>79.63</v>
+        <v>78.43000000000001</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1699,7 +1705,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>59.63</v>
+        <v>58.83</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1712,7 +1718,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>36.89</v>
+        <v>36.17</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1751,7 +1757,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E17</f>
+        <f>MIBGAS_Spot!E18</f>
         <v/>
       </c>
     </row>

</xml_diff>